<commit_message>
untuk navbar static dan update file excel excel bagian
</commit_message>
<xml_diff>
--- a/database/seeders/data/data karyawan 4.xlsx
+++ b/database/seeders/data/data karyawan 4.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BC 20-10-2024\Documents\barcode-project-app\database\seeders\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="480" yWindow="45" windowWidth="22995" windowHeight="10035"/>
   </bookViews>
@@ -17,26 +12,13 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List Karyawan'!$C$2:$F$88</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="177">
   <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nomor Induk Pegawai </t>
-  </si>
-  <si>
-    <t>DEPARTEMEN</t>
-  </si>
-  <si>
-    <t>STATUS KERJA</t>
-  </si>
-  <si>
     <t>JOHANES DJUWANA</t>
   </si>
   <si>
@@ -550,22 +532,34 @@
     <t>Deputi GM Finance &amp; Accounting</t>
   </si>
   <si>
-    <t>JABATAN</t>
-  </si>
-  <si>
-    <t>Nama</t>
+    <t>no</t>
+  </si>
+  <si>
+    <t>nama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nomor induk pegawai </t>
+  </si>
+  <si>
+    <t>departemen</t>
+  </si>
+  <si>
+    <t>jabatan</t>
+  </si>
+  <si>
+    <t>status kerja</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="000###"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -733,8 +727,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="15">
@@ -810,7 +804,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -842,10 +836,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -877,7 +870,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1053,9 +1045,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:GQ90"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="41.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -1066,344 +1058,344 @@
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="12.75" customHeight="1">
       <c r="A1" s="22" t="s">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>1</v>
+        <v>173</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>2</v>
+        <v>174</v>
       </c>
       <c r="E1" s="22" t="s">
         <v>175</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="8" customFormat="1">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C2" s="6">
         <v>990693</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="8" customFormat="1">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C3" s="6">
         <v>960456</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="8" customFormat="1">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C4" s="6">
         <v>990754</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="8" customFormat="1">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F5" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="8" customFormat="1">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C6" s="6">
         <v>970722</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F6" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="8" customFormat="1">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C7" s="6">
         <v>990845</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="8" customFormat="1">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C8" s="6">
         <v>100701</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="8" customFormat="1">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="F9" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="8" customFormat="1">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C10" s="6">
         <v>970663</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="8" customFormat="1">
       <c r="A11" s="4">
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C11" s="6">
         <v>940266</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="8" customFormat="1">
       <c r="A12" s="4">
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C12" s="6">
         <v>990762</v>
       </c>
       <c r="D12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="F12" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="8" customFormat="1">
       <c r="A13" s="4">
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C13" s="6">
         <v>990773</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="8" customFormat="1">
       <c r="A14" s="4">
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F14" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="8" customFormat="1">
       <c r="A15" s="4">
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F15" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="8" customFormat="1">
       <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C16" s="6">
         <v>970640</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:199" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:199">
       <c r="A17" s="4">
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D17" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F17" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -1599,744 +1591,744 @@
       <c r="GP17" s="2"/>
       <c r="GQ17" s="2"/>
     </row>
-    <row r="18" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:199" s="8" customFormat="1">
       <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C18" s="6">
         <v>970740</v>
       </c>
       <c r="D18" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F18" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:199" s="8" customFormat="1">
       <c r="A19" s="4">
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C19" s="6">
         <v>970745</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:199" s="8" customFormat="1">
       <c r="A20" s="4">
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C20" s="11">
         <v>914</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:199" s="8" customFormat="1">
       <c r="A21" s="4">
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C21" s="6">
         <v>990713</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:199" s="8" customFormat="1">
       <c r="A22" s="4">
         <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D22" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F22" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:199" s="8" customFormat="1">
       <c r="A23" s="4">
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C23" s="7">
         <v>140356</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:199" s="8" customFormat="1">
       <c r="A24" s="4">
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C24" s="6">
         <v>940288</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:199" s="8" customFormat="1">
       <c r="A25" s="4">
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:199" s="8" customFormat="1">
       <c r="A26" s="4">
         <v>25</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C26" s="6">
         <v>970726</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:199" s="8" customFormat="1">
       <c r="A27" s="4">
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:199" s="8" customFormat="1">
       <c r="A28" s="4">
         <v>27</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C28" s="7">
         <v>140457</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:199" s="8" customFormat="1">
       <c r="A29" s="4">
         <v>28</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D29" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F29" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:199" s="8" customFormat="1">
       <c r="A30" s="4">
         <v>29</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C30" s="6">
         <v>990820</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:199" s="8" customFormat="1">
       <c r="A31" s="4">
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C31" s="6">
         <v>970673</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:199" s="8" customFormat="1">
       <c r="A32" s="4">
         <v>31</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C32" s="6">
         <v>970737</v>
       </c>
       <c r="D32" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E32" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F32" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" s="8" customFormat="1">
       <c r="A33" s="4">
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C33" s="6">
         <v>940167</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="8" customFormat="1">
       <c r="A34" s="4">
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D34" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E34" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="F34" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" s="8" customFormat="1">
       <c r="A35" s="4">
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="8" customFormat="1">
       <c r="A36" s="4">
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C36" s="6">
         <v>940279</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="8" customFormat="1">
       <c r="A37" s="4">
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E37" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="F37" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" s="8" customFormat="1">
       <c r="A38" s="4">
         <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C38" s="6">
         <v>140865</v>
       </c>
       <c r="D38" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E38" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="F38" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" s="8" customFormat="1">
       <c r="A39" s="4">
         <v>38</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" s="8" customFormat="1">
       <c r="A40" s="4">
         <v>39</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C40" s="6">
         <v>140867</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" s="8" customFormat="1">
       <c r="A41" s="4">
         <v>40</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C41" s="6">
         <v>990695</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" s="8" customFormat="1">
       <c r="A42" s="4">
         <v>41</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C42" s="6">
         <v>960478</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" s="8" customFormat="1">
       <c r="A43" s="4">
         <v>42</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" s="8" customFormat="1">
       <c r="A44" s="4">
         <v>43</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C44" s="6">
         <v>151105</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="8" customFormat="1">
       <c r="A45" s="4">
         <v>44</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" s="8" customFormat="1">
       <c r="A46" s="4">
         <v>45</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C46" s="6">
         <v>960428</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" s="8" customFormat="1">
       <c r="A47" s="4">
         <v>46</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C47" s="6">
         <v>970571</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" s="8" customFormat="1">
       <c r="A48" s="4">
         <v>47</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C48" s="6">
         <v>940122</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="49" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:199" s="8" customFormat="1">
       <c r="A49" s="4">
         <v>48</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C49" s="6">
         <v>990763</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="50" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:199" s="8" customFormat="1">
       <c r="A50" s="4">
         <v>49</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C50" s="6">
         <v>940104</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="51" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:199" s="8" customFormat="1">
       <c r="A51" s="4">
         <v>50</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C51" s="6">
         <v>101101</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E51" s="15" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="52" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:199" s="8" customFormat="1">
       <c r="A52" s="4">
         <v>51</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="53" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:199" s="2" customFormat="1">
       <c r="A53" s="4">
         <v>52</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="54" spans="1:199" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:199">
       <c r="A54" s="4">
         <v>53</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D54" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E54" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="E54" s="17" t="s">
-        <v>26</v>
-      </c>
       <c r="F54" s="5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
@@ -2532,44 +2524,44 @@
       <c r="GP54" s="2"/>
       <c r="GQ54" s="2"/>
     </row>
-    <row r="55" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:199" s="2" customFormat="1">
       <c r="A55" s="4">
         <v>54</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="56" spans="1:199" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:199">
       <c r="A56" s="4">
         <v>55</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C56" s="6">
         <v>960429</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
@@ -2765,24 +2757,24 @@
       <c r="GP56" s="2"/>
       <c r="GQ56" s="2"/>
     </row>
-    <row r="57" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:199">
       <c r="A57" s="4">
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
@@ -2978,24 +2970,24 @@
       <c r="GP57" s="2"/>
       <c r="GQ57" s="2"/>
     </row>
-    <row r="58" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:199">
       <c r="A58" s="4">
         <v>57</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C58" s="6">
         <v>970742</v>
       </c>
       <c r="D58" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E58" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E58" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="F58" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
@@ -3191,24 +3183,24 @@
       <c r="GP58" s="2"/>
       <c r="GQ58" s="2"/>
     </row>
-    <row r="59" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:199">
       <c r="A59" s="4">
         <v>58</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C59" s="6">
         <v>990810</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
@@ -3404,24 +3396,24 @@
       <c r="GP59" s="2"/>
       <c r="GQ59" s="2"/>
     </row>
-    <row r="60" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:199">
       <c r="A60" s="4">
         <v>59</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C60" s="6">
         <v>140758</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
@@ -3617,24 +3609,24 @@
       <c r="GP60" s="2"/>
       <c r="GQ60" s="2"/>
     </row>
-    <row r="61" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:199">
       <c r="A61" s="4">
         <v>60</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C61" s="6">
         <v>970643</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E61" s="15" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
@@ -3830,24 +3822,24 @@
       <c r="GP61" s="2"/>
       <c r="GQ61" s="2"/>
     </row>
-    <row r="62" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:199">
       <c r="A62" s="4">
         <v>61</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C62" s="15">
         <v>990743</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
@@ -4043,364 +4035,364 @@
       <c r="GP62" s="2"/>
       <c r="GQ62" s="2"/>
     </row>
-    <row r="63" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:199" s="2" customFormat="1">
       <c r="A63" s="4">
         <v>62</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="64" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:199" s="2" customFormat="1">
       <c r="A64" s="4">
         <v>63</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C64" s="6">
         <v>990788</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="65" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:199" s="2" customFormat="1">
       <c r="A65" s="4">
         <v>64</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C65" s="6">
         <v>990846</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="66" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:199" s="2" customFormat="1">
       <c r="A66" s="4">
         <v>65</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C66" s="6">
         <v>970557</v>
       </c>
       <c r="D66" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E66" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E66" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="F66" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="67" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:199" s="2" customFormat="1">
       <c r="A67" s="4">
         <v>66</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C67" s="6">
         <v>970714</v>
       </c>
       <c r="D67" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E67" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="F67" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="68" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:199" s="2" customFormat="1">
       <c r="A68" s="4">
         <v>67</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C68" s="6">
         <v>990777</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="69" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:199" s="2" customFormat="1">
       <c r="A69" s="4">
         <v>68</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D69" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E69" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E69" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F69" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="70" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:199" s="2" customFormat="1">
       <c r="A70" s="4">
         <v>69</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C70" s="6">
         <v>970713</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="71" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:199" s="2" customFormat="1">
       <c r="A71" s="4">
         <v>70</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="72" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="72" spans="1:199" s="2" customFormat="1">
       <c r="A72" s="4">
         <v>71</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C72" s="6">
         <v>140859</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="73" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:199" s="2" customFormat="1">
       <c r="A73" s="4">
         <v>72</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C73" s="6">
         <v>990825</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="74" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:199" s="2" customFormat="1">
       <c r="A74" s="4">
         <v>73</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C74" s="9" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="75" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:199" s="2" customFormat="1">
       <c r="A75" s="4">
         <v>74</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C75" s="9" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="76" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:199" s="2" customFormat="1">
       <c r="A76" s="4">
         <v>75</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C76" s="6">
         <v>180302</v>
       </c>
       <c r="D76" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E76" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F76" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="77" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="77" spans="1:199" s="2" customFormat="1">
       <c r="A77" s="4">
         <v>76</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C77" s="9" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="78" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:199" s="2" customFormat="1">
       <c r="A78" s="4">
         <v>77</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="79" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="79" spans="1:199" s="2" customFormat="1">
       <c r="A79" s="4">
         <v>78</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="80" spans="1:199" s="8" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="80" spans="1:199" s="8" customFormat="1">
       <c r="A80" s="4">
         <v>79</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C80" s="6">
         <v>190301</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G80" s="18"/>
       <c r="H80" s="18"/>
@@ -4596,164 +4588,164 @@
       <c r="GP80" s="18"/>
       <c r="GQ80" s="18"/>
     </row>
-    <row r="81" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:199" s="2" customFormat="1">
       <c r="A81" s="4">
         <v>80</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C81" s="7">
         <v>250905</v>
       </c>
       <c r="D81" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E81" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E81" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F81" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="82" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="82" spans="1:199" s="2" customFormat="1">
       <c r="A82" s="4">
         <v>81</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C82" s="9" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="83" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="83" spans="1:199" s="2" customFormat="1">
       <c r="A83" s="4">
         <v>82</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C83" s="7">
         <v>250803</v>
       </c>
       <c r="D83" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E83" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E83" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F83" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="84" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="84" spans="1:199" s="2" customFormat="1">
       <c r="A84" s="4">
         <v>83</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C84" s="7">
         <v>250804</v>
       </c>
       <c r="D84" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E84" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F84" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="85" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="85" spans="1:199" s="2" customFormat="1">
       <c r="A85" s="4">
         <v>84</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C85" s="7">
         <v>251106</v>
       </c>
       <c r="D85" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E85" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E85" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="F85" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="86" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="86" spans="1:199" s="2" customFormat="1">
       <c r="A86" s="4">
         <v>85</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C86" s="7">
         <v>251107</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="87" spans="1:199" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="87" spans="1:199" s="2" customFormat="1">
       <c r="A87" s="4">
         <v>86</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C87" s="6">
         <v>260201</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="88" spans="1:199" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="88" spans="1:199">
       <c r="A88" s="4">
         <v>87</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C88" s="6">
         <v>260302</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
@@ -4949,11 +4941,11 @@
       <c r="GP88" s="2"/>
       <c r="GQ88" s="2"/>
     </row>
-    <row r="89" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:199">
       <c r="D89" s="20"/>
       <c r="E89" s="19"/>
     </row>
-    <row r="90" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:199">
       <c r="B90" s="21"/>
     </row>
   </sheetData>

</xml_diff>